<commit_message>
Updated Pump Upload template with version 1.5 and 3/27/2026
</commit_message>
<xml_diff>
--- a/routes/er_pump_listings.xlsx
+++ b/routes/er_pump_listings.xlsx
@@ -5,12 +5,12 @@
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\dev\hi-er\apps\site\routes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\orig\hi-er\routes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C50805C-8CF5-42C9-80F6-4CA496FD8DD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BAB1220-E02E-4ADA-AABB-07B2EA4C5E67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2232" yWindow="3936" windowWidth="23040" windowHeight="12120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2304" yWindow="2304" windowWidth="23040" windowHeight="12120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Import-Export Sheet" sheetId="1" r:id="rId1"/>
@@ -1255,6 +1255,9 @@
     <xf numFmtId="2" fontId="0" fillId="12" borderId="35" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="2" fontId="0" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1314,9 +1317,6 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="6" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="13" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="89">
@@ -1932,7 +1932,7 @@
       <c r="D2" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="E2" s="124" t="s">
+      <c r="E2" s="104" t="s">
         <v>81</v>
       </c>
       <c r="F2" s="80" t="s">
@@ -1971,26 +1971,26 @@
       <c r="W2" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="X2" s="114" t="s">
+      <c r="X2" s="115" t="s">
         <v>45</v>
       </c>
-      <c r="Y2" s="115"/>
-      <c r="Z2" s="115"/>
-      <c r="AA2" s="115"/>
-      <c r="AB2" s="116"/>
-      <c r="AC2" s="120" t="s">
+      <c r="Y2" s="116"/>
+      <c r="Z2" s="116"/>
+      <c r="AA2" s="116"/>
+      <c r="AB2" s="117"/>
+      <c r="AC2" s="121" t="s">
         <v>46</v>
       </c>
-      <c r="AD2" s="121"/>
-      <c r="AE2" s="121"/>
-      <c r="AF2" s="122"/>
+      <c r="AD2" s="122"/>
+      <c r="AE2" s="122"/>
+      <c r="AF2" s="123"/>
       <c r="AG2" s="33"/>
-      <c r="AH2" s="111" t="s">
+      <c r="AH2" s="112" t="s">
         <v>44</v>
       </c>
-      <c r="AI2" s="112"/>
-      <c r="AJ2" s="112"/>
-      <c r="AK2" s="113"/>
+      <c r="AI2" s="113"/>
+      <c r="AJ2" s="113"/>
+      <c r="AK2" s="114"/>
       <c r="AL2" s="34" t="s">
         <v>38</v>
       </c>
@@ -2033,36 +2033,36 @@
       <c r="Q3" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="R3" s="104" t="s">
+      <c r="R3" s="105" t="s">
         <v>35</v>
       </c>
-      <c r="S3" s="105"/>
-      <c r="T3" s="105"/>
-      <c r="U3" s="105"/>
-      <c r="V3" s="106"/>
+      <c r="S3" s="106"/>
+      <c r="T3" s="106"/>
+      <c r="U3" s="106"/>
+      <c r="V3" s="107"/>
       <c r="W3" s="36"/>
       <c r="X3" s="37"/>
-      <c r="Y3" s="117" t="s">
+      <c r="Y3" s="118" t="s">
         <v>36</v>
       </c>
-      <c r="Z3" s="119"/>
-      <c r="AA3" s="117" t="s">
+      <c r="Z3" s="120"/>
+      <c r="AA3" s="118" t="s">
         <v>37</v>
       </c>
-      <c r="AB3" s="118"/>
-      <c r="AC3" s="123"/>
-      <c r="AD3" s="123"/>
-      <c r="AE3" s="123"/>
-      <c r="AF3" s="123"/>
+      <c r="AB3" s="119"/>
+      <c r="AC3" s="124"/>
+      <c r="AD3" s="124"/>
+      <c r="AE3" s="124"/>
+      <c r="AF3" s="124"/>
       <c r="AG3" s="38"/>
-      <c r="AH3" s="107" t="s">
+      <c r="AH3" s="108" t="s">
         <v>36</v>
       </c>
-      <c r="AI3" s="108"/>
-      <c r="AJ3" s="109" t="s">
+      <c r="AI3" s="109"/>
+      <c r="AJ3" s="110" t="s">
         <v>37</v>
       </c>
-      <c r="AK3" s="110"/>
+      <c r="AK3" s="111"/>
       <c r="AL3" s="39"/>
       <c r="AM3" s="40"/>
       <c r="AN3" s="89"/>
@@ -2369,7 +2369,7 @@
         <v>47</v>
       </c>
       <c r="B1" s="85">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -2377,7 +2377,7 @@
         <v>48</v>
       </c>
       <c r="B2" s="86">
-        <v>45391</v>
+        <v>46108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add  Update pumps with template to Participant Pumps
</commit_message>
<xml_diff>
--- a/routes/er_pump_listings.xlsx
+++ b/routes/er_pump_listings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\orig\hi-er\routes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BAB1220-E02E-4ADA-AABB-07B2EA4C5E67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BECB4B8C-9410-4198-86E1-937337A1515B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2304" yWindow="2304" windowWidth="23040" windowHeight="12120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2328" yWindow="3216" windowWidth="24396" windowHeight="12012" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Import-Export Sheet" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="84">
   <si>
     <t>Nominal Speed</t>
   </si>
@@ -297,6 +297,10 @@
   </si>
   <si>
     <t>Alternative Part Number</t>
+  </si>
+  <si>
+    <t>Only enter data here when updating pumps. 
+Otherwise, only applicable on export.</t>
   </si>
 </sst>
 </file>
@@ -2001,7 +2005,7 @@
         <v>20</v>
       </c>
       <c r="AO2" s="88" t="s">
-        <v>20</v>
+        <v>83</v>
       </c>
       <c r="AP2" s="88" t="s">
         <v>20</v>
@@ -2369,7 +2373,7 @@
         <v>47</v>
       </c>
       <c r="B1" s="85">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -2377,7 +2381,7 @@
         <v>48</v>
       </c>
       <c r="B2" s="86">
-        <v>46108</v>
+        <v>46209</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Revision Note column for Update
</commit_message>
<xml_diff>
--- a/routes/er_pump_listings.xlsx
+++ b/routes/er_pump_listings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\orig\hi-er\routes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BECB4B8C-9410-4198-86E1-937337A1515B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54059514-6307-4746-96CD-5F3A192DA15B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2328" yWindow="3216" windowWidth="24396" windowHeight="12012" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9636" yWindow="2292" windowWidth="20892" windowHeight="12012" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Import-Export Sheet" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="87">
   <si>
     <t>Nominal Speed</t>
   </si>
@@ -244,9 +244,6 @@
     <t>Not displayed on the label</t>
   </si>
   <si>
-    <t>Displayed on the label</t>
-  </si>
-  <si>
     <t>Equipment Category
 of rated pump</t>
   </si>
@@ -299,8 +296,49 @@
     <t>Alternative Part Number</t>
   </si>
   <si>
-    <t>Only enter data here when updating pumps. 
+    <t>Revision Note</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Not displayed on the label
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Do not change for an update</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Displayed on the label
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Do not change for an update</t>
+    </r>
+  </si>
+  <si>
+    <t>Enter the Rating ID when updating pumps. 
 Otherwise, only applicable on export.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only Enter data here when updating pumps.
+Otherwise, not applicable </t>
   </si>
 </sst>
 </file>
@@ -460,7 +498,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="37">
+  <borders count="38">
     <border>
       <left/>
       <right/>
@@ -890,6 +928,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -982,7 +1035,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="125">
+  <cellXfs count="128">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
@@ -1260,6 +1313,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="13" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1749,7 +1811,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR9"/>
+  <dimension ref="A1:AS9"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.8984375" style="1" customWidth="1"/>
@@ -1787,9 +1849,10 @@
     <col min="39" max="42" width="18.59765625" style="56" customWidth="1"/>
     <col min="43" max="43" width="11" style="94"/>
     <col min="44" max="44" width="11" style="95"/>
+    <col min="45" max="45" width="21.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:44" s="3" customFormat="1" ht="78" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:45" s="3" customFormat="1" ht="78" x14ac:dyDescent="0.3">
       <c r="A1" s="57" t="s">
         <v>49</v>
       </c>
@@ -1803,10 +1866,10 @@
         <v>51</v>
       </c>
       <c r="E1" s="81" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F1" s="59" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G1" s="59" t="s">
         <v>52</v>
@@ -1917,27 +1980,30 @@
         <v>59</v>
       </c>
       <c r="AQ1" s="96" t="s">
+        <v>78</v>
+      </c>
+      <c r="AR1" s="97" t="s">
         <v>79</v>
       </c>
-      <c r="AR1" s="97" t="s">
-        <v>80</v>
+      <c r="AS1" s="107" t="s">
+        <v>82</v>
       </c>
     </row>
-    <row r="2" spans="1:44" s="7" customFormat="1" ht="109.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:45" s="7" customFormat="1" ht="109.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
-        <v>64</v>
+        <v>83</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>64</v>
       </c>
       <c r="E2" s="104" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F2" s="80" t="s">
         <v>41</v>
@@ -1975,26 +2041,26 @@
       <c r="W2" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="X2" s="115" t="s">
+      <c r="X2" s="118" t="s">
         <v>45</v>
       </c>
-      <c r="Y2" s="116"/>
-      <c r="Z2" s="116"/>
-      <c r="AA2" s="116"/>
-      <c r="AB2" s="117"/>
-      <c r="AC2" s="121" t="s">
+      <c r="Y2" s="119"/>
+      <c r="Z2" s="119"/>
+      <c r="AA2" s="119"/>
+      <c r="AB2" s="120"/>
+      <c r="AC2" s="124" t="s">
         <v>46</v>
       </c>
-      <c r="AD2" s="122"/>
-      <c r="AE2" s="122"/>
-      <c r="AF2" s="123"/>
+      <c r="AD2" s="125"/>
+      <c r="AE2" s="125"/>
+      <c r="AF2" s="126"/>
       <c r="AG2" s="33"/>
-      <c r="AH2" s="112" t="s">
+      <c r="AH2" s="115" t="s">
         <v>44</v>
       </c>
-      <c r="AI2" s="113"/>
-      <c r="AJ2" s="113"/>
-      <c r="AK2" s="114"/>
+      <c r="AI2" s="116"/>
+      <c r="AJ2" s="116"/>
+      <c r="AK2" s="117"/>
       <c r="AL2" s="34" t="s">
         <v>38</v>
       </c>
@@ -2005,7 +2071,7 @@
         <v>20</v>
       </c>
       <c r="AO2" s="88" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="AP2" s="88" t="s">
         <v>20</v>
@@ -2016,8 +2082,11 @@
       <c r="AR2" s="99" t="s">
         <v>20</v>
       </c>
+      <c r="AS2" s="88" t="s">
+        <v>86</v>
+      </c>
     </row>
-    <row r="3" spans="1:44" s="12" customFormat="1" ht="78.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:45" s="12" customFormat="1" ht="78.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="8"/>
       <c r="B3" s="9"/>
       <c r="C3" s="82"/>
@@ -2037,36 +2106,36 @@
       <c r="Q3" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="R3" s="105" t="s">
+      <c r="R3" s="108" t="s">
         <v>35</v>
       </c>
-      <c r="S3" s="106"/>
-      <c r="T3" s="106"/>
-      <c r="U3" s="106"/>
-      <c r="V3" s="107"/>
+      <c r="S3" s="109"/>
+      <c r="T3" s="109"/>
+      <c r="U3" s="109"/>
+      <c r="V3" s="110"/>
       <c r="W3" s="36"/>
       <c r="X3" s="37"/>
-      <c r="Y3" s="118" t="s">
+      <c r="Y3" s="121" t="s">
         <v>36</v>
       </c>
-      <c r="Z3" s="120"/>
-      <c r="AA3" s="118" t="s">
+      <c r="Z3" s="123"/>
+      <c r="AA3" s="121" t="s">
         <v>37</v>
       </c>
-      <c r="AB3" s="119"/>
-      <c r="AC3" s="124"/>
-      <c r="AD3" s="124"/>
-      <c r="AE3" s="124"/>
-      <c r="AF3" s="124"/>
+      <c r="AB3" s="122"/>
+      <c r="AC3" s="127"/>
+      <c r="AD3" s="127"/>
+      <c r="AE3" s="127"/>
+      <c r="AF3" s="127"/>
       <c r="AG3" s="38"/>
-      <c r="AH3" s="108" t="s">
+      <c r="AH3" s="111" t="s">
         <v>36</v>
       </c>
-      <c r="AI3" s="109"/>
-      <c r="AJ3" s="110" t="s">
+      <c r="AI3" s="112"/>
+      <c r="AJ3" s="113" t="s">
         <v>37</v>
       </c>
-      <c r="AK3" s="111"/>
+      <c r="AK3" s="114"/>
       <c r="AL3" s="39"/>
       <c r="AM3" s="40"/>
       <c r="AN3" s="89"/>
@@ -2074,8 +2143,9 @@
       <c r="AP3" s="89"/>
       <c r="AQ3" s="100"/>
       <c r="AR3" s="101"/>
+      <c r="AS3" s="105"/>
     </row>
-    <row r="4" spans="1:44" s="17" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:45" s="17" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="14"/>
       <c r="B4" s="14"/>
       <c r="C4" s="83"/>
@@ -2120,11 +2190,12 @@
       <c r="AP4" s="89"/>
       <c r="AQ4" s="102"/>
       <c r="AR4" s="103"/>
+      <c r="AS4" s="106"/>
     </row>
-    <row r="5" spans="1:44" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:45" x14ac:dyDescent="0.3">
       <c r="AK5" s="55"/>
     </row>
-    <row r="9" spans="1:44" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:45" x14ac:dyDescent="0.3">
       <c r="AJ9" s="29" t="s">
         <v>28</v>
       </c>
@@ -2271,7 +2342,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="F6" s="92" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -2284,7 +2355,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F8">
         <v>4</v>
@@ -2292,7 +2363,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F9">
         <v>5</v>
@@ -2300,7 +2371,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F10">
         <v>6</v>
@@ -2313,17 +2384,17 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="92" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F14" s="92" t="s">
         <v>22</v>
@@ -2331,23 +2402,23 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F16" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bulk update pumps to Beta (#29)
* Add  Update pumps with template to Participant Pumps

* Add Revision Note column for Update
</commit_message>
<xml_diff>
--- a/routes/er_pump_listings.xlsx
+++ b/routes/er_pump_listings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\orig\hi-er\routes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BAB1220-E02E-4ADA-AABB-07B2EA4C5E67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54059514-6307-4746-96CD-5F3A192DA15B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2304" yWindow="2304" windowWidth="23040" windowHeight="12120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9636" yWindow="2292" windowWidth="20892" windowHeight="12012" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Import-Export Sheet" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="87">
   <si>
     <t>Nominal Speed</t>
   </si>
@@ -244,9 +244,6 @@
     <t>Not displayed on the label</t>
   </si>
   <si>
-    <t>Displayed on the label</t>
-  </si>
-  <si>
     <t>Equipment Category
 of rated pump</t>
   </si>
@@ -297,6 +294,51 @@
   </si>
   <si>
     <t>Alternative Part Number</t>
+  </si>
+  <si>
+    <t>Revision Note</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Not displayed on the label
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Do not change for an update</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Displayed on the label
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Do not change for an update</t>
+    </r>
+  </si>
+  <si>
+    <t>Enter the Rating ID when updating pumps. 
+Otherwise, only applicable on export.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only Enter data here when updating pumps.
+Otherwise, not applicable </t>
   </si>
 </sst>
 </file>
@@ -456,7 +498,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="37">
+  <borders count="38">
     <border>
       <left/>
       <right/>
@@ -886,6 +928,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -978,7 +1035,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="125">
+  <cellXfs count="128">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
@@ -1256,6 +1313,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="13" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1745,7 +1811,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR9"/>
+  <dimension ref="A1:AS9"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.8984375" style="1" customWidth="1"/>
@@ -1783,9 +1849,10 @@
     <col min="39" max="42" width="18.59765625" style="56" customWidth="1"/>
     <col min="43" max="43" width="11" style="94"/>
     <col min="44" max="44" width="11" style="95"/>
+    <col min="45" max="45" width="21.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:44" s="3" customFormat="1" ht="78" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:45" s="3" customFormat="1" ht="78" x14ac:dyDescent="0.3">
       <c r="A1" s="57" t="s">
         <v>49</v>
       </c>
@@ -1799,10 +1866,10 @@
         <v>51</v>
       </c>
       <c r="E1" s="81" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F1" s="59" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G1" s="59" t="s">
         <v>52</v>
@@ -1913,27 +1980,30 @@
         <v>59</v>
       </c>
       <c r="AQ1" s="96" t="s">
+        <v>78</v>
+      </c>
+      <c r="AR1" s="97" t="s">
         <v>79</v>
       </c>
-      <c r="AR1" s="97" t="s">
-        <v>80</v>
+      <c r="AS1" s="107" t="s">
+        <v>82</v>
       </c>
     </row>
-    <row r="2" spans="1:44" s="7" customFormat="1" ht="109.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:45" s="7" customFormat="1" ht="109.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
-        <v>64</v>
+        <v>83</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>64</v>
       </c>
       <c r="E2" s="104" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F2" s="80" t="s">
         <v>41</v>
@@ -1971,26 +2041,26 @@
       <c r="W2" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="X2" s="115" t="s">
+      <c r="X2" s="118" t="s">
         <v>45</v>
       </c>
-      <c r="Y2" s="116"/>
-      <c r="Z2" s="116"/>
-      <c r="AA2" s="116"/>
-      <c r="AB2" s="117"/>
-      <c r="AC2" s="121" t="s">
+      <c r="Y2" s="119"/>
+      <c r="Z2" s="119"/>
+      <c r="AA2" s="119"/>
+      <c r="AB2" s="120"/>
+      <c r="AC2" s="124" t="s">
         <v>46</v>
       </c>
-      <c r="AD2" s="122"/>
-      <c r="AE2" s="122"/>
-      <c r="AF2" s="123"/>
+      <c r="AD2" s="125"/>
+      <c r="AE2" s="125"/>
+      <c r="AF2" s="126"/>
       <c r="AG2" s="33"/>
-      <c r="AH2" s="112" t="s">
+      <c r="AH2" s="115" t="s">
         <v>44</v>
       </c>
-      <c r="AI2" s="113"/>
-      <c r="AJ2" s="113"/>
-      <c r="AK2" s="114"/>
+      <c r="AI2" s="116"/>
+      <c r="AJ2" s="116"/>
+      <c r="AK2" s="117"/>
       <c r="AL2" s="34" t="s">
         <v>38</v>
       </c>
@@ -2001,7 +2071,7 @@
         <v>20</v>
       </c>
       <c r="AO2" s="88" t="s">
-        <v>20</v>
+        <v>85</v>
       </c>
       <c r="AP2" s="88" t="s">
         <v>20</v>
@@ -2012,8 +2082,11 @@
       <c r="AR2" s="99" t="s">
         <v>20</v>
       </c>
+      <c r="AS2" s="88" t="s">
+        <v>86</v>
+      </c>
     </row>
-    <row r="3" spans="1:44" s="12" customFormat="1" ht="78.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:45" s="12" customFormat="1" ht="78.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="8"/>
       <c r="B3" s="9"/>
       <c r="C3" s="82"/>
@@ -2033,36 +2106,36 @@
       <c r="Q3" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="R3" s="105" t="s">
+      <c r="R3" s="108" t="s">
         <v>35</v>
       </c>
-      <c r="S3" s="106"/>
-      <c r="T3" s="106"/>
-      <c r="U3" s="106"/>
-      <c r="V3" s="107"/>
+      <c r="S3" s="109"/>
+      <c r="T3" s="109"/>
+      <c r="U3" s="109"/>
+      <c r="V3" s="110"/>
       <c r="W3" s="36"/>
       <c r="X3" s="37"/>
-      <c r="Y3" s="118" t="s">
+      <c r="Y3" s="121" t="s">
         <v>36</v>
       </c>
-      <c r="Z3" s="120"/>
-      <c r="AA3" s="118" t="s">
+      <c r="Z3" s="123"/>
+      <c r="AA3" s="121" t="s">
         <v>37</v>
       </c>
-      <c r="AB3" s="119"/>
-      <c r="AC3" s="124"/>
-      <c r="AD3" s="124"/>
-      <c r="AE3" s="124"/>
-      <c r="AF3" s="124"/>
+      <c r="AB3" s="122"/>
+      <c r="AC3" s="127"/>
+      <c r="AD3" s="127"/>
+      <c r="AE3" s="127"/>
+      <c r="AF3" s="127"/>
       <c r="AG3" s="38"/>
-      <c r="AH3" s="108" t="s">
+      <c r="AH3" s="111" t="s">
         <v>36</v>
       </c>
-      <c r="AI3" s="109"/>
-      <c r="AJ3" s="110" t="s">
+      <c r="AI3" s="112"/>
+      <c r="AJ3" s="113" t="s">
         <v>37</v>
       </c>
-      <c r="AK3" s="111"/>
+      <c r="AK3" s="114"/>
       <c r="AL3" s="39"/>
       <c r="AM3" s="40"/>
       <c r="AN3" s="89"/>
@@ -2070,8 +2143,9 @@
       <c r="AP3" s="89"/>
       <c r="AQ3" s="100"/>
       <c r="AR3" s="101"/>
+      <c r="AS3" s="105"/>
     </row>
-    <row r="4" spans="1:44" s="17" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:45" s="17" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="14"/>
       <c r="B4" s="14"/>
       <c r="C4" s="83"/>
@@ -2116,11 +2190,12 @@
       <c r="AP4" s="89"/>
       <c r="AQ4" s="102"/>
       <c r="AR4" s="103"/>
+      <c r="AS4" s="106"/>
     </row>
-    <row r="5" spans="1:44" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:45" x14ac:dyDescent="0.3">
       <c r="AK5" s="55"/>
     </row>
-    <row r="9" spans="1:44" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:45" x14ac:dyDescent="0.3">
       <c r="AJ9" s="29" t="s">
         <v>28</v>
       </c>
@@ -2267,7 +2342,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="F6" s="92" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -2280,7 +2355,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F8">
         <v>4</v>
@@ -2288,7 +2363,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F9">
         <v>5</v>
@@ -2296,7 +2371,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F10">
         <v>6</v>
@@ -2309,17 +2384,17 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="92" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F14" s="92" t="s">
         <v>22</v>
@@ -2327,23 +2402,23 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F16" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -2369,7 +2444,7 @@
         <v>47</v>
       </c>
       <c r="B1" s="85">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -2377,7 +2452,7 @@
         <v>48</v>
       </c>
       <c r="B2" s="86">
-        <v>46108</v>
+        <v>46209</v>
       </c>
     </row>
   </sheetData>

</xml_diff>